<commit_message>
Feldcheck von JNK: 1 bestätigt, 0 fehlen, 0 verschoben, 0 neu
</commit_message>
<xml_diff>
--- a/karte/out/Wangerooge_West_Landmarken_v1.xlsx
+++ b/karte/out/Wangerooge_West_Landmarken_v1.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Landmarken" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pfade prüfen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Übersicht" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Landmarken" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pfade prüfen" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Landmarken'!$A$1:$M$885</definedName>
@@ -44229,7 +44229,7 @@
       </c>
       <c r="F869" s="3" t="inlineStr">
         <is>
-          <t>OSM + aloeus.de: Zum Westen 32</t>
+          <t>OSM + aloeus.de: Zum Westen 32 + Feldbegehung JNK 13.10.2026</t>
         </is>
       </c>
       <c r="G869" s="9" t="n">

</xml_diff>

<commit_message>
App im Glas-Design, kürzere Texte; Legende nach Linien, Flächen, Punkten
- Karte füllt den Bildschirm; Kopfleiste, Objektkarte und Menüs schweben als
  Glasflächen darüber (iOS-Systemschrift, scharf statt Handschrift-Webfont)
- Kopfleiste: Name + Fortschritt, Symbole für GPS / Liste / Mehr; Folgen-Knopf
  und Zoom als Glasknöpfe rechts
- Objektkarte: Titel, ein Satz „Was du suchst“, Ort und Grund als kurze Zeilen,
  große Knöpfe Stimmt / Fehlt / Woanders
- Mehr: gruppierte Abschnitte (Senden, Karte, Anzeigen, Legende, Hilfe, Briefkasten)
- Alle Texte gekürzt (App, Einführung, Objekttexte)
- Dunkelmodus mit kräftigerem Glas
- Kartenlegende: Linien, Flächen, Karte | Orientierungspunkte, Landmarken,
  Ausstattung; Ebenenliste im PDF-Export und Filter in der App gleich sortiert

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011qSH9gX535fj8mWz8WvNAQ
</commit_message>
<xml_diff>
--- a/karte/out/Wangerooge_West_Landmarken_v1.xlsx
+++ b/karte/out/Wangerooge_West_Landmarken_v1.xlsx
@@ -45187,11 +45187,7 @@
           <t>footway</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Belag dirt, Länge 345 m, Luftbild sichtbar 29%</t>
-        </is>
-      </c>
+      <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45209,11 +45205,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Belag dirt, Länge 100 m, Luftbild sichtbar 15%</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45231,11 +45223,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Belag grass, Länge 34 m, Luftbild sichtbar 20%</t>
-        </is>
-      </c>
+      <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45253,11 +45241,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Belag grass, Länge 191 m, Luftbild sichtbar 35%</t>
-        </is>
-      </c>
+      <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45275,11 +45259,7 @@
           <t>footway</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Belag unbekannt, Länge 46 m, Luftbild sichtbar 37%</t>
-        </is>
-      </c>
+      <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45297,11 +45277,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Belag dirt, Länge 38 m, Luftbild sichtbar 23%</t>
-        </is>
-      </c>
+      <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45319,11 +45295,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Belag sand, Länge 1308 m, Luftbild sichtbar 31%</t>
-        </is>
-      </c>
+      <c r="C8" s="3" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45341,11 +45313,7 @@
           <t>footway</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Belag unbekannt, Länge 72 m, Luftbild sichtbar 40%</t>
-        </is>
-      </c>
+      <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45363,11 +45331,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Belag sand, Länge 6 m, Luftbild sichtbar 43%</t>
-        </is>
-      </c>
+      <c r="C10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45385,11 +45349,7 @@
           <t>footway</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Belag unbekannt, Länge 51 m, Luftbild sichtbar 31%</t>
-        </is>
-      </c>
+      <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45407,11 +45367,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Belag grass, Länge 97 m, Luftbild sichtbar 5%</t>
-        </is>
-      </c>
+      <c r="C12" s="3" t="inlineStr"/>
       <c r="D12" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45429,11 +45385,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Belag sand, Länge 50 m, Luftbild sichtbar 2%</t>
-        </is>
-      </c>
+      <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45451,11 +45403,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Belag dirt, Länge 24 m, Luftbild sichtbar 24%</t>
-        </is>
-      </c>
+      <c r="C14" s="3" t="inlineStr"/>
       <c r="D14" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45473,11 +45421,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Belag dirt, Länge 54 m, Luftbild sichtbar 35%</t>
-        </is>
-      </c>
+      <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45495,11 +45439,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Belag sand, Länge 155 m, Luftbild sichtbar 34%</t>
-        </is>
-      </c>
+      <c r="C16" s="3" t="inlineStr"/>
       <c r="D16" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45517,11 +45457,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Belag dirt, Länge 67 m, Luftbild sichtbar 19%</t>
-        </is>
-      </c>
+      <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45539,11 +45475,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Belag dirt, Länge 254 m, Luftbild sichtbar 41%</t>
-        </is>
-      </c>
+      <c r="C18" s="3" t="inlineStr"/>
       <c r="D18" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45561,11 +45493,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Belag grass, Länge 53 m, Luftbild sichtbar 7%</t>
-        </is>
-      </c>
+      <c r="C19" s="3" t="inlineStr"/>
       <c r="D19" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45583,11 +45511,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Belag unbekannt, Länge 78 m, Luftbild sichtbar 35%</t>
-        </is>
-      </c>
+      <c r="C20" s="3" t="inlineStr"/>
       <c r="D20" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45605,11 +45529,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Belag grass, Länge 146 m, Luftbild sichtbar 29%</t>
-        </is>
-      </c>
+      <c r="C21" s="3" t="inlineStr"/>
       <c r="D21" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45627,11 +45547,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Belag dirt, Länge 218 m, Luftbild sichtbar 42%</t>
-        </is>
-      </c>
+      <c r="C22" s="3" t="inlineStr"/>
       <c r="D22" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45649,11 +45565,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Belag unbekannt, Länge 163 m, Luftbild sichtbar 42%</t>
-        </is>
-      </c>
+      <c r="C23" s="3" t="inlineStr"/>
       <c r="D23" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45671,11 +45583,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Belag sand, Länge 26 m, Luftbild sichtbar 8%</t>
-        </is>
-      </c>
+      <c r="C24" s="3" t="inlineStr"/>
       <c r="D24" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>
@@ -45693,11 +45601,7 @@
           <t>path</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Belag grass, Länge 56 m, Luftbild sichtbar 34%</t>
-        </is>
-      </c>
+      <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr">
         <is>
           <t>OSM; im Luftbild kaum sichtbar</t>

</xml_diff>